<commit_message>
update tracking table of augmenting path
</commit_message>
<xml_diff>
--- a/26fall/1870/Note/w1s1_augmenting_path_find.xlsx
+++ b/26fall/1870/Note/w1s1_augmenting_path_find.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vcboy1\Desktop\大学\课程\Leeds\26fall\1870\Note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CC2A4AF-46F1-4B4A-BF25-638D1C38BDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64D22A7-1F4F-4B02-9619-4B0CE085DE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="8085" windowWidth="14295" windowHeight="7095" xr2:uid="{56E2E4A5-E210-4D13-A903-8FC1FF3E665A}"/>
+    <workbookView xWindow="315" yWindow="7545" windowWidth="14295" windowHeight="7680" xr2:uid="{56E2E4A5-E210-4D13-A903-8FC1FF3E665A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="112">
   <si>
     <t>Matching</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -451,7 +451,26 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2,y,6,z</t>
+    <t>v</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v-&gt;3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>loop8</t>
+  </si>
+  <si>
+    <t>5,u,3,v</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3,z</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2,3,4,5,6,x,y,z,u,v</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1323,9 +1342,7 @@
       <c r="E26" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F26" s="3">
-        <v>2</v>
-      </c>
+      <c r="F26" s="3"/>
       <c r="G26" s="3" t="s">
         <v>77</v>
       </c>
@@ -1373,9 +1390,7 @@
       <c r="E28" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F28" s="3">
-        <v>5</v>
-      </c>
+      <c r="F28" s="3"/>
       <c r="G28" s="3" t="s">
         <v>74</v>
       </c>
@@ -1495,8 +1510,8 @@
       <c r="B33" s="3">
         <v>2.5</v>
       </c>
-      <c r="C33" s="6">
-        <v>3</v>
+      <c r="C33" s="6" t="s">
+        <v>110</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>104</v>
@@ -1510,28 +1525,41 @@
       <c r="G33" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="H33" s="3">
-        <v>2</v>
-      </c>
-      <c r="I33" s="3">
-        <v>2</v>
-      </c>
-      <c r="J33" s="5" t="s">
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F34" s="3">
+        <v>3</v>
+      </c>
+      <c r="G34" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="K33" s="3"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="H34" s="3" t="s">
+        <v>106</v>
+      </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
+      <c r="K34" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>

</xml_diff>